<commit_message>
update ailog, code, data
</commit_message>
<xml_diff>
--- a/ai_logs/Nguyên_AI_Log.xlsx
+++ b/ai_logs/Nguyên_AI_Log.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ADMIN\Downloads\SUM26\labl\Food_delivery\ai_logs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BCA8FBC3-9741-4B40-A99A-86F524E3FFB7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{203A5EE5-78E2-492A-AC69-3FEE70DDF38B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="1. Metadata &amp; Summary" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="343" uniqueCount="261">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="395" uniqueCount="299">
   <si>
     <t>DETAILED AI AUDIT LOG</t>
   </si>
@@ -844,6 +844,135 @@
   </si>
   <si>
     <t>AI lưu feedback của Customer vào List&lt;String&gt; in-memory và khẳng định Restaurant có thể 'đọc được những phản hồi chính xác này từ khách' qua chức năng Quản lý phản hồi — ngụ ý feedback tồn tại lâu dài như dữ liệu thật.</t>
+  </si>
+  <si>
+    <t>LockMechanism.java đã được viết sẵn với 4 enum: NO_LOCK, SYNCHRONIZED, FILE_LOCK, OPTIMISTIC. Cần hiểu rõ từng cơ chế trước khi viết báo cáo phân tích và chuẩn bị trả lời GV về lý do chọn Optimistic Locking làm cơ chế chính cho Food Delivery.</t>
+  </si>
+  <si>
+    <t>AI đọc file và giải thích 4 cơ chế: (1) NO_LOCK — không bảo vệ, nhanh nhất, dễ Race Condition khi 2 tài xế nhận cùng 1 đơn; (2) SYNCHRONIZED — Java keyword/ReentrantLock, chỉ hiệu quả trên 1 JVM, không dùng được cho Distributed System; (3) FILE_LOCK — dùng java.nio.channels.FileLock của OS, hiệu quả giữa các process trên cùng 1 máy nhưng chậm do I/O; (4) OPTIMISTIC — đọc version khi lấy data, kiểm tra version trước khi ghi, ném lỗi nếu version đã thay đổi (người khác đã cập nhật trước). Kết luận: Optimistic phù hợp nhất cho hệ thống đọc nhiều hơn ghi.</t>
+  </si>
+  <si>
+    <t>Critical Thinking: AI giải thích SYNCHRONIZED 'không hiệu quả cho Distributed System' — đúng về lý thuyết, nhưng project này chạy trên 1 JVM duy nhất (single process, multi-thread). Trong phạm vi LAB211, SYNCHRONIZED vẫn ngăn được Race Condition hoàn toàn; hạn chế Distributed chỉ liên quan khi triển khai production thực tế, không phải bối cảnh đề bài.
+Contextualization: GV có thể hỏi 'Tại sao không dùng SYNCHRONIZED thay vì OPTIMISTIC?' — cần câu trả lời cân bằng: SYNCHRONIZED đúng cho single JVM, OPTIMISTIC đúng hơn khi muốn mô phỏng hành vi database thực tế (version column).
+Creative Synthesis: Bổ sung vào bảng so sánh 4 cơ chế trong báo cáo thêm cột 'Phạm vi áp dụng' (Single JVM / Single Machine / Distributed) để GV thấy nhóm hiểu context, không chỉ học vẹt lý thuyết.
+Decision: Dùng toàn bộ giải thích AI làm nội dung báo cáo; bổ sung thêm cột 'Phạm vi' và câu chú thích 'Trong LAB211, project chạy single JVM nên cả SYNCHRONIZED và OPTIMISTIC đều ngăn được Race Condition — OPTIMISTIC được chọn vì mô phỏng sát hành vi database thực tế hơn'.</t>
+  </si>
+  <si>
+    <t>Bảng so sánh 4 cơ chế trong báo cáo (5 cột: Tên / Phương thức / Phạm vi / Ưu điểm / Nhược điểm) + câu chú thích về single JVM context</t>
+  </si>
+  <si>
+    <t>Sau khi chạy Simulator, console in ra bảng kết quả với các con số Success/Failed/Throughput. Cần chứng minh với GV rằng các con số này không phải 'bịa ra' mà có thể verify độc lập bằng file CSV — đây là yêu cầu thực nghiệm (empirical proof) của đề bài.</t>
+  </si>
+  <si>
+    <t>AI đọc 3 file (MainApplication, SimulatorController, SimulatorView) và đề xuất 4 cách verify: (1) Tổng Success + Failed = TOTAL_CUSTOMERS=100 luôn đúng; (2) Mở menu_items.csv kiểm tra stock âm sau NO_LOCK (Oversell proof); (3) Mở orders.csv tìm driver_id xuất hiện ≥2 lần với status CONFIRMED (Overload proof); (4) Console đọc lại trực tiếp từ simulation_runs.csv chứ không phải biến RAM — mở CSV đối chiếu từng dòng.</t>
+  </si>
+  <si>
+    <t>Critical Thinking: Cách verify (4) của AI mô tả đúng nhưng cần làm rõ một điểm quan trọng: printLockComparisonTableFromFile() đọc lại từ file là đúng — nhưng nếu file CSV bị ghi sai (bug trong saveSimulationResult()), console sẽ vẫn hiển thị số sai mà verify bằng cách so sánh console với CSV cũng không phát hiện được. Verify thực sự cần đếm thủ công trong orders.csv và menu_items.csv.
+Contextualization: GV thường yêu cầu 'mở file CSV lên cho tôi xem' trong buổi demo — cần chuẩn bị sẵn 3 file CSV sau mỗi kịch bản chạy, không để lẫn giữa các lần chạy (NO_LOCK vs SYNCHRONIZED output khác nhau).
+Creative Synthesis: Xây dựng quy trình verify 3 bước cho buổi demo: Bước 1 — chạy NO_LOCK và lưu screenshot console; Bước 2 — mở menu_items.csv đếm số dòng có stockQty &lt; 0; Bước 3 — mở orders.csv dùng Excel filter driver_id và đếm CONFIRMED trùng. Ba bước này independent nhau và không phụ thuộc vào console.
+Decision: Chuẩn bị 'Verify Checklist' 3 bước cho buổi demo; chụp screenshot CSV làm evidence trong báo cáo; không chỉ dùng console screenshot.</t>
+  </si>
+  <si>
+    <t>Verify checklist 3 bước + screenshot menu_items.csv (stockQty âm sau NO_LOCK) + screenshot orders.csv (driver_id trùng CONFIRMED) + so sánh với console output</t>
+  </si>
+  <si>
+    <t>Cần tìm đúng file source code chứa logic của từng phần Simulator để phân công thành viên báo cáo và để bản thân hiểu rõ flow code trước khi GV hỏi chi tiết implementation. AI đọc LockMechanism.java nhưng cần tìm file thực thi logic.</t>
+  </si>
+  <si>
+    <t>AI grep codebase, đọc drivers.csv để hiểu data structure, chỉ ra 4 file chính: (1) SimulatorController.java — runSimulation() tạo 100 CustomerThread + 20 DispatchThread, vòng lặp 4 loại Lock, detectOversellItems(), detectDriverOverload(); (2) MenuItemRepository.java — validateAndDeductStockAtomically() là 'trái tim' xử lý đụng độ kho hàng với 3 nhánh synchronized/FileLock/version check; (3) ReportView.java — saveSimulationResult() ghi CSV, printLockComparisonTableFromFile() đọc và vẽ bảng console; (4) data/ folder — menu_items.csv, orders.csv, simulation_runs.csv.</t>
+  </si>
+  <si>
+    <t>Critical Thinking: AI chỉ ra 4 file nhưng không đề cập đến CustomerThread.java và DispatchThread.java — đây là 2 file quan trọng nhất để hiểu RACE CONDITION xảy ra ở đâu (CustomerThread gọi validateAndDeductStockAtomically, DispatchThread gọi hàm gán tài xế). Nếu không đọc 2 file này, không thể giải thích được tại sao NO_LOCK gây lỗi ở cả 2 loại: Oversell (kho âm) và Overload (tài xế trùng).
+Contextualization: GV thường hỏi 'Race Condition xảy ra cụ thể ở đoạn code nào?' — câu trả lời phải chỉ được đúng method trong CustomerThread/DispatchThread, không chỉ nói chung chung.
+Creative Synthesis: Tự đọc thêm CustomerThread.java và DispatchThread.java để bổ sung vào sơ đồ luồng (flow diagram): Thread → gọi Repository method → Lock check → read CSV → check condition → write CSV → release Lock.
+Decision: Vẽ flow diagram đầy đủ 6 bước cho mỗi cơ chế Lock; phân công mỗi thành viên giải thích 1-2 cơ chế với flow diagram tương ứng trong buổi báo cáo.</t>
+  </si>
+  <si>
+    <t>Flow diagram 6 bước (Thread → Repository → Lock → Read → Check → Write) cho 4 cơ chế Lock + danh sách 6 file chính (thêm CustomerThread và DispatchThread)</t>
+  </si>
+  <si>
+    <t>Sau khi chạy Simulator với SYNCHRONIZED và FILE_LOCK, kết quả console luôn hiện Success = 50, Failed = 50. Nhóm không chắc đây là hành vi đúng hay Simulator đang bị bug — cần xác nhận trước khi báo cáo.</t>
+  </si>
+  <si>
+    <t>AI đọc MenuItemRepository.java và giải thích: đây là hành vi đúng, không phải bug. SYNCHRONIZED và FILE_LOCK là Pessimistic Locking — ép 100 luồng xếp hàng tuần tự. 50 người đầu lấy được lock thấy stock &gt; 0 → mua thành công. Người thứ 51 lấy lock thấy stock = 0 → từ chối (Failed). Kết quả: Success=50 = stock ban đầu, Failed=50 = 100-50. Đề xuất test: đổi TOTAL_CUSTOMERS=120 sẽ ra Success=50, Failed=70 (không còn bằng nhau) để chứng minh logic đúng.</t>
+  </si>
+  <si>
+    <t>Critical Thinking: Giải thích của AI hoàn toàn đúng và đầy đủ về mặt lý thuyết. Tuy nhiên có một điểm tinh tế cần bổ sung cho báo cáo: với OPTIMISTIC, kết quả cũng phải là Success=50, Failed=50 nếu cơ chế hoạt động đúng — nhưng nếu OPTIMISTIC bị implement sai (ví dụ version check không atomic), Success có thể &gt; 50 (tức vẫn còn Oversell dù dùng Optimistic). Việc OPTIMISTIC cũng cho Success=50 là bằng chứng cơ chế hoạt động đúng, không phải trùng hợp.
+Contextualization: GV có thể hỏi 'Thế NO_LOCK cho Success bao nhiêu?' — câu trả lời đúng là Success &gt; 50 (thường 70-100 tùy race condition) và stockQty trong CSV bị âm. Đây mới là điểm phân biệt NO_LOCK với 3 cơ chế còn lại.
+Creative Synthesis: Áp dụng test AI đề xuất: chạy TOTAL_CUSTOMERS=120 để verify; ghi rõ trong báo cáo 'Success=50 với mọi Locking mechanism ≠ bug; nó chứng minh cả 3 cơ chế (SYNCHRONIZED/FILE_LOCK/OPTIMISTIC) đều bảo vệ đúng stock limit'.
+Decision: Chạy test TOTAL_CUSTOMERS=120 để có thêm bằng chứng; bổ sung vào báo cáo bảng kết quả với 2 kịch bản (100 và 120 customers) để chứng minh tính nhất quán của kết quả.</t>
+  </si>
+  <si>
+    <t>Console screenshot TOTAL_CUSTOMERS=100 (Success=50, Failed=50) + TOTAL_CUSTOMERS=120 (Success=50, Failed=70) cho SYNCHRONIZED và FILE_LOCK + ghi chú 'Success=50 là stock limit, không phải bug'</t>
+  </si>
+  <si>
+    <t>Bảng console in cột 'THPUT(d/s)' nhưng nhóm không rõ công thức tính throughput và cách đọc con số này để so sánh hiệu năng giữa 4 cơ chế Lock trong báo cáo. Đây là chỉ số định lượng quan trọng để trả lời câu hỏi nghiên cứu (RQ) về hiệu năng.</t>
+  </si>
+  <si>
+    <t>AI đọc SimulationRun.java, tìm đúng dòng code công thức: throughput = durationMs &gt; 0 ? (totalSuccess * 1000.0 / durationMs) : 0. Giải thích: totalSuccess (đơn thành công) × 1000 ÷ durationMs (ms) = đơn/giây. Ví dụ: 50 success ÷ 500ms × 1000 = 100 đơn/giây. Dự đoán thứ tự throughput: NO_LOCK cao nhất (không chờ), OPTIMISTIC nhì, FILE_LOCK thấp nhất (I/O latency).</t>
+  </si>
+  <si>
+    <t>Critical Thinking: Dự đoán thứ tự throughput của AI (NO_LOCK &gt; OPTIMISTIC &gt; SYNCHRONIZED &gt; FILE_LOCK) là đúng về lý thuyết, nhưng trong thực tế benchmark với 100 threads trên máy cá nhân: (a) SYNCHRONIZED và OPTIMISTIC có thể cho throughput gần tương đương vì cả hai đều phải đọc/ghi file CSV tuần tự — bottleneck thực sự là I/O disk, không phải lock overhead; (b) FILE_LOCK chậm nhất vì gọi OS-level file lock, nhưng mức chênh lệch phụ thuộc vào SSD vs HDD.
+Contextualization: GV sẽ hỏi 'Tại sao OPTIMISTIC không nhanh hơn SYNCHRONIZED nhiều như lý thuyết?' — câu trả lời: trong project này cả hai đều phải gọi readAll() và saveAll() trên file CSV, I/O là bottleneck chung, lock overhead nhỏ hơn I/O latency nên throughput không chênh nhiều.
+Creative Synthesis: Ghi rõ trong báo cáo 2 tầng: (1) Throughput lý thuyết (theo lock mechanism), (2) Throughput thực tế (bị giới hạn bởi I/O bottleneck của CSV-based storage). Thêm ghi chú: 'Với database thực (MySQL/PostgreSQL), khoảng cách OPTIMISTIC vs SYNCHRONIZED sẽ rõ hơn nhiều'.
+Decision: Dùng công thức AI cung cấp làm nội dung giải thích trong báo cáo; bổ sung phần nhận xét về I/O bottleneck và so sánh lý thuyết vs thực nghiệm để thể hiện nhóm hiểu giới hạn của mô hình CSV.</t>
+  </si>
+  <si>
+    <t>Dòng code công thức throughput trong SimulationRun.java (dòng 46/62) + bảng console 4 cơ chế Lock với cột THPUT(d/s) + nhận xét về I/O bottleneck trong báo cáo</t>
+  </si>
+  <si>
+    <t>"giải thích phần 4 cơ chế lock" (kèm LockMechanism.java)</t>
+  </si>
+  <si>
+    <t>"làm sao để chứng minh con số hiển thị trên console là đúng?"</t>
+  </si>
+  <si>
+    <t>"code của phần này ở đâu"</t>
+  </si>
+  <si>
+    <t>"tại sao synchronized và file lock luôn có success = failed"</t>
+  </si>
+  <si>
+    <t>"through put tính sao"</t>
+  </si>
+  <si>
+    <t>014</t>
+  </si>
+  <si>
+    <t>015</t>
+  </si>
+  <si>
+    <t>016</t>
+  </si>
+  <si>
+    <t>017</t>
+  </si>
+  <si>
+    <t>018</t>
+  </si>
+  <si>
+    <t>AI khẳng định SYNCHRONIZED 'không hiệu quả' và 'không còn tác dụng' cho hệ thống Food Delivery vì giới hạn Single JVM — ngụ ý OPTIMISTIC là lựa chọn duy nhất đúng cho project này.</t>
+  </si>
+  <si>
+    <t>Project LAB211 chạy hoàn toàn trên 1 JVM (single process, multi-thread). Trong phạm vi này, SYNCHRONIZED ngăn Race Condition 100% và cho kết quả Success=50 giống hệt OPTIMISTIC. Hạn chế 'Distributed System' của SYNCHRONIZED chỉ liên quan khi triển khai production thực tế trên nhiều server — không áp dụng cho ngữ cảnh LAB211.</t>
+  </si>
+  <si>
+    <t>Phân tích kết quả Simulator: SYNCHRONIZED cho Success=50 giống OPTIMISTIC, chứng minh cả hai đều hoạt động đúng trong phạm vi single JVM. Đối chiếu với lý thuyết concurrency: synchronized keyword đủ để bảo vệ shared resource trong multi-thread single process.</t>
+  </si>
+  <si>
+    <t>Bổ sung cột 'Phạm vi áp dụng' vào bảng so sánh 4 cơ chế; thêm câu chú thích: 'Trong LAB211 (single JVM), cả SYNCHRONIZED và OPTIMISTIC đều ngăn được Race Condition — OPTIMISTIC được chọn vì mô phỏng sát hành vi database version column hơn, không phải vì SYNCHRONIZED sai'.</t>
+  </si>
+  <si>
+    <t>AI dự đoán thứ tự throughput NO_LOCK &gt; OPTIMISTIC &gt; SYNCHRONIZED &gt; FILE_LOCK như một quy luật chắc chắn, ngụ ý OPTIMISTIC sẽ nhanh hơn SYNCHRONIZED rõ rệt trong kết quả benchmark của project.</t>
+  </si>
+  <si>
+    <t>Trong project dùng CSV file làm storage, bottleneck thực sự là I/O disk (readAll() và saveAll() gọi cho mọi cơ chế Lock). Lock overhead (synchronized vs version check) nhỏ hơn nhiều so với I/O latency nên OPTIMISTIC và SYNCHRONIZED thường cho throughput gần tương đương trong benchmark thực tế. Khoảng cách lý thuyết chỉ rõ khi dùng in-memory storage hoặc database thực.</t>
+  </si>
+  <si>
+    <t>Chạy Simulator và quan sát cột THPUT(d/s): SYNCHRONIZED và OPTIMISTIC cho throughput chênh lệch nhỏ hơn dự đoán của AI. Phân tích nguồn gốc: cả hai đều gọi readAll()/saveAll() — I/O là common bottleneck.</t>
+  </si>
+  <si>
+    <t>Bổ sung vào báo cáo phần 'Nhận xét thực nghiệm': throughput bị giới hạn bởi I/O bottleneck của CSV storage; thêm ghi chú 'Với database thực (MySQL), khoảng cách OPTIMISTIC vs SYNCHRONIZED sẽ rõ hơn nhiều do in-memory index'; phân biệt rõ throughput lý thuyết vs thực nghiệm trong bảng so sánh.</t>
   </si>
 </sst>
 </file>
@@ -853,7 +982,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="21" x14ac:knownFonts="1">
+  <fonts count="28" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -894,19 +1023,6 @@
       <i/>
       <sz val="10"/>
       <color rgb="FF666666"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="16"/>
-      <color rgb="FFFF0000"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <b/>
-      <i/>
-      <sz val="10"/>
-      <color rgb="FFFF0000"/>
       <name val="Calibri"/>
     </font>
     <font>
@@ -952,11 +1068,6 @@
     </font>
     <font>
       <b/>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <b/>
       <sz val="9"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
@@ -971,8 +1082,74 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color rgb="FF2E75B6"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color rgb="FFFF0000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <i/>
+      <sz val="9"/>
+      <color rgb="FFFF0000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="12">
+  <fills count="13">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1032,6 +1209,12 @@
         <fgColor rgb="FFFFF2CC"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="4">
     <border>
@@ -1086,7 +1269,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="52">
+  <cellXfs count="57">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1111,117 +1294,132 @@
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="14" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="10" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="16" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="11" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="3" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="10" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="11" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="11" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="11" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="9" borderId="3" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="11" borderId="3" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="6" borderId="3" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="11" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="11" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="11" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="20" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="11" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="11" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="11" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="9" borderId="3" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="11" borderId="3" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="12" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1536,14 +1734,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A1" s="45" t="s">
+      <c r="A1" s="34" t="s">
         <v>44</v>
       </c>
-      <c r="B1" s="44"/>
-      <c r="C1" s="44"/>
-      <c r="D1" s="44"/>
-      <c r="E1" s="44"/>
-      <c r="F1" s="44"/>
+      <c r="B1" s="35"/>
+      <c r="C1" s="35"/>
+      <c r="D1" s="35"/>
+      <c r="E1" s="35"/>
+      <c r="F1" s="35"/>
     </row>
     <row r="3" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
@@ -1795,28 +1993,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A1" s="45" t="s">
+      <c r="A1" s="34" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="44"/>
-      <c r="C1" s="44"/>
-      <c r="D1" s="44"/>
-      <c r="E1" s="44"/>
-      <c r="F1" s="44"/>
-      <c r="G1" s="44"/>
-      <c r="H1" s="44"/>
+      <c r="B1" s="35"/>
+      <c r="C1" s="35"/>
+      <c r="D1" s="35"/>
+      <c r="E1" s="35"/>
+      <c r="F1" s="35"/>
+      <c r="G1" s="35"/>
+      <c r="H1" s="35"/>
     </row>
     <row r="2" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="43" t="s">
+      <c r="A2" s="36" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="44"/>
-      <c r="C2" s="44"/>
-      <c r="D2" s="44"/>
-      <c r="E2" s="44"/>
-      <c r="F2" s="44"/>
-      <c r="G2" s="44"/>
-      <c r="H2" s="44"/>
+      <c r="B2" s="35"/>
+      <c r="C2" s="35"/>
+      <c r="D2" s="35"/>
+      <c r="E2" s="35"/>
+      <c r="F2" s="35"/>
+      <c r="G2" s="35"/>
+      <c r="H2" s="35"/>
     </row>
     <row r="3" spans="1:8" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="6" t="s">
@@ -1845,7 +2043,7 @@
       </c>
     </row>
     <row r="4" spans="1:8" ht="109.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="37" t="s">
+      <c r="A4" s="32" t="s">
         <v>10</v>
       </c>
       <c r="B4" s="20" t="s">
@@ -1866,12 +2064,12 @@
       <c r="G4" s="22" t="s">
         <v>22</v>
       </c>
-      <c r="H4" s="40" t="s">
+      <c r="H4" s="33" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="109.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="37" t="s">
+      <c r="A5" s="32" t="s">
         <v>13</v>
       </c>
       <c r="B5" s="23" t="s">
@@ -1897,7 +2095,7 @@
       </c>
     </row>
     <row r="6" spans="1:8" ht="109.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="37" t="s">
+      <c r="A6" s="32" t="s">
         <v>16</v>
       </c>
       <c r="B6" s="23" t="s">
@@ -1923,7 +2121,7 @@
       </c>
     </row>
     <row r="7" spans="1:8" ht="151.80000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="37" t="s">
+      <c r="A7" s="32" t="s">
         <v>18</v>
       </c>
       <c r="B7" s="28" t="s">
@@ -1949,7 +2147,7 @@
       </c>
     </row>
     <row r="8" spans="1:8" ht="130.19999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="37" t="s">
+      <c r="A8" s="32" t="s">
         <v>24</v>
       </c>
       <c r="B8" s="23" t="s">
@@ -1975,7 +2173,7 @@
       </c>
     </row>
     <row r="9" spans="1:8" ht="249" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="37" t="s">
+      <c r="A9" s="32" t="s">
         <v>30</v>
       </c>
       <c r="B9" s="20" t="s">
@@ -2001,7 +2199,7 @@
       </c>
     </row>
     <row r="10" spans="1:8" ht="205.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="37" t="s">
+      <c r="A10" s="32" t="s">
         <v>37</v>
       </c>
       <c r="B10" s="28" t="s">
@@ -2027,7 +2225,7 @@
       </c>
     </row>
     <row r="11" spans="1:8" ht="230.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="37" t="s">
+      <c r="A11" s="32" t="s">
         <v>212</v>
       </c>
       <c r="B11" s="23" t="s">
@@ -2053,7 +2251,7 @@
       </c>
     </row>
     <row r="12" spans="1:8" ht="200.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="37" t="s">
+      <c r="A12" s="32" t="s">
         <v>228</v>
       </c>
       <c r="B12" s="20" t="s">
@@ -2079,7 +2277,7 @@
       </c>
     </row>
     <row r="13" spans="1:8" ht="202.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="37" t="s">
+      <c r="A13" s="32" t="s">
         <v>249</v>
       </c>
       <c r="B13" s="20" t="s">
@@ -2105,7 +2303,7 @@
       </c>
     </row>
     <row r="14" spans="1:8" ht="200.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="37" t="s">
+      <c r="A14" s="32" t="s">
         <v>250</v>
       </c>
       <c r="B14" s="23" t="s">
@@ -2131,7 +2329,7 @@
       </c>
     </row>
     <row r="15" spans="1:8" ht="196.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="37" t="s">
+      <c r="A15" s="32" t="s">
         <v>251</v>
       </c>
       <c r="B15" s="28" t="s">
@@ -2157,7 +2355,7 @@
       </c>
     </row>
     <row r="16" spans="1:8" ht="222.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="37" t="s">
+      <c r="A16" s="32" t="s">
         <v>252</v>
       </c>
       <c r="B16" s="20" t="s">
@@ -2182,55 +2380,135 @@
         <v>223</v>
       </c>
     </row>
-    <row r="17" spans="1:8" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="7"/>
-      <c r="B17" s="7"/>
-      <c r="C17" s="7"/>
-      <c r="D17" s="7"/>
-      <c r="E17" s="7"/>
-      <c r="F17" s="7"/>
-      <c r="G17" s="7"/>
-      <c r="H17" s="7"/>
-    </row>
-    <row r="18" spans="1:8" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="7"/>
-      <c r="B18" s="7"/>
-      <c r="C18" s="7"/>
-      <c r="D18" s="7"/>
-      <c r="E18" s="7"/>
-      <c r="F18" s="7"/>
-      <c r="G18" s="7"/>
-      <c r="H18" s="7"/>
-    </row>
-    <row r="19" spans="1:8" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="7"/>
-      <c r="B19" s="7"/>
-      <c r="C19" s="7"/>
-      <c r="D19" s="7"/>
-      <c r="E19" s="7"/>
-      <c r="F19" s="7"/>
-      <c r="G19" s="7"/>
-      <c r="H19" s="7"/>
-    </row>
-    <row r="20" spans="1:8" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="7"/>
-      <c r="B20" s="7"/>
-      <c r="C20" s="7"/>
-      <c r="D20" s="7"/>
-      <c r="E20" s="7"/>
-      <c r="F20" s="7"/>
-      <c r="G20" s="7"/>
-      <c r="H20" s="7"/>
-    </row>
-    <row r="21" spans="1:8" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="7"/>
-      <c r="B21" s="7"/>
-      <c r="C21" s="7"/>
-      <c r="D21" s="7"/>
-      <c r="E21" s="7"/>
-      <c r="F21" s="7"/>
-      <c r="G21" s="7"/>
-      <c r="H21" s="7"/>
+    <row r="17" spans="1:8" ht="208.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="32" t="s">
+        <v>286</v>
+      </c>
+      <c r="B17" s="20" t="s">
+        <v>11</v>
+      </c>
+      <c r="C17" s="21" t="s">
+        <v>38</v>
+      </c>
+      <c r="D17" s="22" t="s">
+        <v>261</v>
+      </c>
+      <c r="E17" s="22" t="s">
+        <v>281</v>
+      </c>
+      <c r="F17" s="22" t="s">
+        <v>262</v>
+      </c>
+      <c r="G17" s="22" t="s">
+        <v>263</v>
+      </c>
+      <c r="H17" s="22" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" ht="187.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="32" t="s">
+        <v>287</v>
+      </c>
+      <c r="B18" s="28" t="s">
+        <v>17</v>
+      </c>
+      <c r="C18" s="24" t="s">
+        <v>31</v>
+      </c>
+      <c r="D18" s="25" t="s">
+        <v>265</v>
+      </c>
+      <c r="E18" s="25" t="s">
+        <v>282</v>
+      </c>
+      <c r="F18" s="25" t="s">
+        <v>266</v>
+      </c>
+      <c r="G18" s="25" t="s">
+        <v>267</v>
+      </c>
+      <c r="H18" s="25" t="s">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" ht="175.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="32" t="s">
+        <v>288</v>
+      </c>
+      <c r="B19" s="23" t="s">
+        <v>14</v>
+      </c>
+      <c r="C19" s="26" t="s">
+        <v>12</v>
+      </c>
+      <c r="D19" s="27" t="s">
+        <v>269</v>
+      </c>
+      <c r="E19" s="27" t="s">
+        <v>283</v>
+      </c>
+      <c r="F19" s="27" t="s">
+        <v>270</v>
+      </c>
+      <c r="G19" s="27" t="s">
+        <v>271</v>
+      </c>
+      <c r="H19" s="27" t="s">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" ht="217.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A20" s="32" t="s">
+        <v>289</v>
+      </c>
+      <c r="B20" s="28" t="s">
+        <v>17</v>
+      </c>
+      <c r="C20" s="21" t="s">
+        <v>31</v>
+      </c>
+      <c r="D20" s="22" t="s">
+        <v>273</v>
+      </c>
+      <c r="E20" s="22" t="s">
+        <v>284</v>
+      </c>
+      <c r="F20" s="22" t="s">
+        <v>274</v>
+      </c>
+      <c r="G20" s="22" t="s">
+        <v>275</v>
+      </c>
+      <c r="H20" s="22" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" ht="213.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A21" s="32" t="s">
+        <v>290</v>
+      </c>
+      <c r="B21" s="23" t="s">
+        <v>14</v>
+      </c>
+      <c r="C21" s="24" t="s">
+        <v>15</v>
+      </c>
+      <c r="D21" s="25" t="s">
+        <v>277</v>
+      </c>
+      <c r="E21" s="25" t="s">
+        <v>285</v>
+      </c>
+      <c r="F21" s="25" t="s">
+        <v>278</v>
+      </c>
+      <c r="G21" s="25" t="s">
+        <v>279</v>
+      </c>
+      <c r="H21" s="25" t="s">
+        <v>280</v>
+      </c>
     </row>
     <row r="22" spans="1:8" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="7"/>
@@ -2264,451 +2542,476 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:F41"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="12" customWidth="1"/>
-    <col min="2" max="2" width="22" style="39" customWidth="1"/>
-    <col min="3" max="6" width="30" customWidth="1"/>
+    <col min="1" max="1" width="12" style="43" customWidth="1"/>
+    <col min="2" max="2" width="22" style="43" customWidth="1"/>
+    <col min="3" max="6" width="30" style="43" customWidth="1"/>
+    <col min="7" max="16384" width="8.88671875" style="43"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A1" s="48" t="s">
+      <c r="A1" s="47" t="s">
         <v>85</v>
       </c>
-      <c r="B1" s="47"/>
-      <c r="C1" s="47"/>
-      <c r="D1" s="47"/>
-      <c r="E1" s="47"/>
-      <c r="F1" s="47"/>
+      <c r="B1" s="48"/>
+      <c r="C1" s="48"/>
+      <c r="D1" s="48"/>
+      <c r="E1" s="48"/>
+      <c r="F1" s="48"/>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A2" s="46" t="s">
+      <c r="A2" s="49" t="s">
         <v>86</v>
       </c>
-      <c r="B2" s="47"/>
-      <c r="C2" s="47"/>
-      <c r="D2" s="47"/>
-      <c r="E2" s="47"/>
-      <c r="F2" s="47"/>
+      <c r="B2" s="48"/>
+      <c r="C2" s="48"/>
+      <c r="D2" s="48"/>
+      <c r="E2" s="48"/>
+      <c r="F2" s="48"/>
     </row>
     <row r="3" spans="1:6" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="6" t="s">
+      <c r="A3" s="50" t="s">
         <v>87</v>
       </c>
-      <c r="B3" s="6" t="s">
+      <c r="B3" s="50" t="s">
         <v>88</v>
       </c>
-      <c r="C3" s="6" t="s">
+      <c r="C3" s="50" t="s">
         <v>89</v>
       </c>
-      <c r="D3" s="6" t="s">
+      <c r="D3" s="50" t="s">
         <v>90</v>
       </c>
-      <c r="E3" s="6" t="s">
+      <c r="E3" s="50" t="s">
         <v>91</v>
       </c>
-      <c r="F3" s="6" t="s">
+      <c r="F3" s="50" t="s">
         <v>92</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="35" t="s">
+      <c r="A4" s="51" t="s">
         <v>13</v>
       </c>
-      <c r="B4" s="26" t="s">
+      <c r="B4" s="38" t="s">
         <v>94</v>
       </c>
-      <c r="C4" s="41" t="s">
+      <c r="C4" s="39" t="s">
         <v>95</v>
       </c>
-      <c r="D4" s="41" t="s">
+      <c r="D4" s="39" t="s">
         <v>96</v>
       </c>
-      <c r="E4" s="41" t="s">
+      <c r="E4" s="39" t="s">
         <v>97</v>
       </c>
-      <c r="F4" s="41" t="s">
+      <c r="F4" s="39" t="s">
         <v>98</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="36" t="s">
+      <c r="A5" s="52" t="s">
         <v>16</v>
       </c>
-      <c r="B5" s="38" t="s">
+      <c r="B5" s="40" t="s">
         <v>99</v>
       </c>
-      <c r="C5" s="42" t="s">
+      <c r="C5" s="41" t="s">
         <v>100</v>
       </c>
-      <c r="D5" s="42" t="s">
+      <c r="D5" s="41" t="s">
         <v>101</v>
       </c>
-      <c r="E5" s="42" t="s">
+      <c r="E5" s="41" t="s">
         <v>102</v>
       </c>
-      <c r="F5" s="42" t="s">
+      <c r="F5" s="41" t="s">
         <v>103</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="35" t="s">
+      <c r="A6" s="51" t="s">
         <v>18</v>
       </c>
-      <c r="B6" s="26" t="s">
+      <c r="B6" s="38" t="s">
         <v>94</v>
       </c>
-      <c r="C6" s="41" t="s">
+      <c r="C6" s="39" t="s">
         <v>104</v>
       </c>
-      <c r="D6" s="41" t="s">
+      <c r="D6" s="39" t="s">
         <v>105</v>
       </c>
-      <c r="E6" s="41" t="s">
+      <c r="E6" s="39" t="s">
         <v>106</v>
       </c>
-      <c r="F6" s="41" t="s">
+      <c r="F6" s="39" t="s">
         <v>107</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="99" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="35" t="s">
+      <c r="A7" s="51" t="s">
         <v>24</v>
       </c>
-      <c r="B7" s="26" t="s">
+      <c r="B7" s="38" t="s">
         <v>94</v>
       </c>
-      <c r="C7" s="41" t="s">
+      <c r="C7" s="39" t="s">
         <v>213</v>
       </c>
-      <c r="D7" s="41" t="s">
+      <c r="D7" s="39" t="s">
         <v>214</v>
       </c>
-      <c r="E7" s="41" t="s">
+      <c r="E7" s="39" t="s">
         <v>215</v>
       </c>
-      <c r="F7" s="41" t="s">
+      <c r="F7" s="39" t="s">
         <v>216</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="148.19999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="36" t="s">
+      <c r="A8" s="52" t="s">
         <v>37</v>
       </c>
-      <c r="B8" s="38" t="s">
+      <c r="B8" s="40" t="s">
         <v>99</v>
       </c>
-      <c r="C8" s="42" t="s">
+      <c r="C8" s="41" t="s">
         <v>217</v>
       </c>
-      <c r="D8" s="42" t="s">
+      <c r="D8" s="41" t="s">
         <v>218</v>
       </c>
-      <c r="E8" s="42" t="s">
+      <c r="E8" s="41" t="s">
         <v>219</v>
       </c>
-      <c r="F8" s="42" t="s">
+      <c r="F8" s="41" t="s">
         <v>220</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="127.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="35" t="s">
+      <c r="A9" s="51" t="s">
         <v>251</v>
       </c>
-      <c r="B9" s="51" t="s">
+      <c r="B9" s="38" t="s">
         <v>94</v>
       </c>
-      <c r="C9" s="27" t="s">
+      <c r="C9" s="39" t="s">
         <v>260</v>
       </c>
-      <c r="D9" s="27" t="s">
+      <c r="D9" s="39" t="s">
         <v>259</v>
       </c>
-      <c r="E9" s="27" t="s">
+      <c r="E9" s="39" t="s">
         <v>258</v>
       </c>
-      <c r="F9" s="27" t="s">
+      <c r="F9" s="39" t="s">
         <v>257</v>
       </c>
     </row>
     <row r="10" spans="1:6" ht="136.80000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="36" t="s">
+      <c r="A10" s="52" t="s">
         <v>252</v>
       </c>
-      <c r="B10" s="50" t="s">
+      <c r="B10" s="40" t="s">
         <v>99</v>
       </c>
-      <c r="C10" s="31" t="s">
+      <c r="C10" s="41" t="s">
         <v>256</v>
       </c>
-      <c r="D10" s="31" t="s">
+      <c r="D10" s="41" t="s">
         <v>255</v>
       </c>
-      <c r="E10" s="31" t="s">
+      <c r="E10" s="41" t="s">
         <v>254</v>
       </c>
-      <c r="F10" s="31" t="s">
+      <c r="F10" s="41" t="s">
         <v>253</v>
       </c>
     </row>
-    <row r="11" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="7"/>
-      <c r="B11" s="9"/>
-      <c r="C11" s="7"/>
-      <c r="D11" s="7"/>
-      <c r="E11" s="7"/>
-      <c r="F11" s="7"/>
-    </row>
-    <row r="12" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="7"/>
-      <c r="B12" s="9"/>
-      <c r="C12" s="7"/>
-      <c r="D12" s="7"/>
-      <c r="E12" s="7"/>
-      <c r="F12" s="7"/>
+    <row r="11" spans="1:6" ht="133.19999999999999" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="55" t="s">
+        <v>286</v>
+      </c>
+      <c r="B11" s="56" t="s">
+        <v>99</v>
+      </c>
+      <c r="C11" s="53" t="s">
+        <v>291</v>
+      </c>
+      <c r="D11" s="53" t="s">
+        <v>292</v>
+      </c>
+      <c r="E11" s="53" t="s">
+        <v>293</v>
+      </c>
+      <c r="F11" s="53" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" ht="141" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="55" t="s">
+        <v>290</v>
+      </c>
+      <c r="B12" s="56" t="s">
+        <v>99</v>
+      </c>
+      <c r="C12" s="53" t="s">
+        <v>295</v>
+      </c>
+      <c r="D12" s="53" t="s">
+        <v>296</v>
+      </c>
+      <c r="E12" s="53" t="s">
+        <v>297</v>
+      </c>
+      <c r="F12" s="53" t="s">
+        <v>298</v>
+      </c>
     </row>
     <row r="13" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="7"/>
-      <c r="B13" s="9"/>
-      <c r="C13" s="7"/>
-      <c r="D13" s="7"/>
-      <c r="E13" s="7"/>
-      <c r="F13" s="7"/>
+      <c r="A13" s="42"/>
+      <c r="B13" s="42"/>
+      <c r="C13" s="42"/>
+      <c r="D13" s="42"/>
+      <c r="E13" s="42"/>
+      <c r="F13" s="42"/>
     </row>
     <row r="14" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="7"/>
-      <c r="B14" s="9"/>
-      <c r="C14" s="7"/>
-      <c r="D14" s="7"/>
-      <c r="E14" s="7"/>
-      <c r="F14" s="7"/>
+      <c r="A14" s="42"/>
+      <c r="B14" s="42"/>
+      <c r="C14" s="42"/>
+      <c r="D14" s="42"/>
+      <c r="E14" s="42"/>
+      <c r="F14" s="42"/>
     </row>
     <row r="15" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="7"/>
-      <c r="B15" s="9"/>
-      <c r="C15" s="7"/>
-      <c r="D15" s="7"/>
-      <c r="E15" s="7"/>
-      <c r="F15" s="7"/>
+      <c r="A15" s="42"/>
+      <c r="B15" s="42"/>
+      <c r="C15" s="42"/>
+      <c r="D15" s="42"/>
+      <c r="E15" s="42"/>
+      <c r="F15" s="42"/>
     </row>
     <row r="16" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="7"/>
-      <c r="B16" s="9"/>
-      <c r="C16" s="7"/>
-      <c r="D16" s="7"/>
-      <c r="E16" s="7"/>
-      <c r="F16" s="7"/>
+      <c r="A16" s="42"/>
+      <c r="B16" s="42"/>
+      <c r="C16" s="42"/>
+      <c r="D16" s="42"/>
+      <c r="E16" s="42"/>
+      <c r="F16" s="42"/>
     </row>
     <row r="17" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="7"/>
-      <c r="B17" s="9"/>
-      <c r="C17" s="7"/>
-      <c r="D17" s="7"/>
-      <c r="E17" s="7"/>
-      <c r="F17" s="7"/>
+      <c r="A17" s="42"/>
+      <c r="B17" s="42"/>
+      <c r="C17" s="42"/>
+      <c r="D17" s="42"/>
+      <c r="E17" s="42"/>
+      <c r="F17" s="42"/>
     </row>
     <row r="18" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="7"/>
-      <c r="B18" s="9"/>
-      <c r="C18" s="7"/>
-      <c r="D18" s="7"/>
-      <c r="E18" s="7"/>
-      <c r="F18" s="7"/>
+      <c r="A18" s="42"/>
+      <c r="B18" s="42"/>
+      <c r="C18" s="42"/>
+      <c r="D18" s="42"/>
+      <c r="E18" s="42"/>
+      <c r="F18" s="42"/>
     </row>
     <row r="19" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="7"/>
-      <c r="B19" s="9"/>
-      <c r="C19" s="7"/>
-      <c r="D19" s="7"/>
-      <c r="E19" s="7"/>
-      <c r="F19" s="7"/>
+      <c r="A19" s="42"/>
+      <c r="B19" s="42"/>
+      <c r="C19" s="42"/>
+      <c r="D19" s="42"/>
+      <c r="E19" s="42"/>
+      <c r="F19" s="42"/>
     </row>
     <row r="20" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="7"/>
-      <c r="B20" s="9"/>
-      <c r="C20" s="7"/>
-      <c r="D20" s="7"/>
-      <c r="E20" s="7"/>
-      <c r="F20" s="7"/>
+      <c r="A20" s="42"/>
+      <c r="B20" s="42"/>
+      <c r="C20" s="42"/>
+      <c r="D20" s="42"/>
+      <c r="E20" s="42"/>
+      <c r="F20" s="42"/>
     </row>
     <row r="21" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="7"/>
-      <c r="B21" s="9"/>
-      <c r="C21" s="7"/>
-      <c r="D21" s="7"/>
-      <c r="E21" s="7"/>
-      <c r="F21" s="7"/>
+      <c r="A21" s="42"/>
+      <c r="B21" s="42"/>
+      <c r="C21" s="42"/>
+      <c r="D21" s="42"/>
+      <c r="E21" s="42"/>
+      <c r="F21" s="42"/>
     </row>
     <row r="22" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="7"/>
-      <c r="B22" s="9"/>
-      <c r="C22" s="7"/>
-      <c r="D22" s="7"/>
-      <c r="E22" s="7"/>
-      <c r="F22" s="7"/>
+      <c r="A22" s="42"/>
+      <c r="B22" s="42"/>
+      <c r="C22" s="42"/>
+      <c r="D22" s="42"/>
+      <c r="E22" s="42"/>
+      <c r="F22" s="42"/>
     </row>
     <row r="23" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="7"/>
-      <c r="B23" s="9"/>
-      <c r="C23" s="7"/>
-      <c r="D23" s="7"/>
-      <c r="E23" s="7"/>
-      <c r="F23" s="7"/>
+      <c r="A23" s="42"/>
+      <c r="B23" s="42"/>
+      <c r="C23" s="42"/>
+      <c r="D23" s="42"/>
+      <c r="E23" s="42"/>
+      <c r="F23" s="42"/>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A24" s="7"/>
-      <c r="B24" s="9"/>
-      <c r="C24" s="7"/>
-      <c r="D24" s="7"/>
-      <c r="E24" s="7"/>
-      <c r="F24" s="7"/>
+      <c r="A24" s="42"/>
+      <c r="B24" s="42"/>
+      <c r="C24" s="42"/>
+      <c r="D24" s="42"/>
+      <c r="E24" s="42"/>
+      <c r="F24" s="42"/>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A25" s="7"/>
-      <c r="B25" s="9"/>
-      <c r="C25" s="7"/>
-      <c r="D25" s="7"/>
-      <c r="E25" s="7"/>
-      <c r="F25" s="7"/>
+      <c r="A25" s="42"/>
+      <c r="B25" s="42"/>
+      <c r="C25" s="42"/>
+      <c r="D25" s="42"/>
+      <c r="E25" s="42"/>
+      <c r="F25" s="42"/>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A26" s="7"/>
-      <c r="B26" s="9"/>
-      <c r="C26" s="7"/>
-      <c r="D26" s="7"/>
-      <c r="E26" s="7"/>
-      <c r="F26" s="7"/>
+      <c r="A26" s="42"/>
+      <c r="B26" s="42"/>
+      <c r="C26" s="42"/>
+      <c r="D26" s="42"/>
+      <c r="E26" s="42"/>
+      <c r="F26" s="42"/>
     </row>
     <row r="29" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="31" spans="1:6" ht="28.8" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="32" spans="1:6" ht="28.8" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A32" s="1" t="s">
+    <row r="32" spans="1:6" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A32" s="54" t="s">
         <v>108</v>
       </c>
     </row>
     <row r="33" spans="1:6" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A33" s="10" t="s">
+      <c r="A33" s="44" t="s">
         <v>109</v>
       </c>
-      <c r="B33" s="17" t="s">
+      <c r="B33" s="44" t="s">
         <v>110</v>
       </c>
-      <c r="C33" s="10" t="s">
+      <c r="C33" s="44" t="s">
         <v>111</v>
       </c>
     </row>
     <row r="34" spans="1:6" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A34" s="7" t="s">
+      <c r="A34" s="42" t="s">
         <v>93</v>
       </c>
-      <c r="B34" s="9" t="s">
+      <c r="B34" s="42" t="s">
         <v>112</v>
       </c>
-      <c r="C34" s="7" t="s">
+      <c r="C34" s="42" t="s">
         <v>113</v>
       </c>
     </row>
     <row r="35" spans="1:6" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="7" t="s">
+      <c r="A35" s="42" t="s">
         <v>99</v>
       </c>
-      <c r="B35" s="9" t="s">
+      <c r="B35" s="42" t="s">
         <v>114</v>
       </c>
-      <c r="C35" s="7" t="s">
+      <c r="C35" s="42" t="s">
         <v>115</v>
       </c>
     </row>
     <row r="36" spans="1:6" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A36" s="7" t="s">
+      <c r="A36" s="42" t="s">
         <v>94</v>
       </c>
-      <c r="B36" s="9" t="s">
+      <c r="B36" s="42" t="s">
         <v>116</v>
       </c>
-      <c r="C36" s="7" t="s">
+      <c r="C36" s="42" t="s">
         <v>117</v>
       </c>
     </row>
     <row r="37" spans="1:6" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A37" s="7" t="s">
+      <c r="A37" s="42" t="s">
         <v>118</v>
       </c>
-      <c r="B37" s="9" t="s">
+      <c r="B37" s="42" t="s">
         <v>119</v>
       </c>
-      <c r="C37" s="7" t="s">
+      <c r="C37" s="42" t="s">
         <v>120</v>
       </c>
     </row>
     <row r="38" spans="1:6" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A38" s="7" t="s">
+      <c r="A38" s="42" t="s">
         <v>121</v>
       </c>
-      <c r="B38" s="9" t="s">
+      <c r="B38" s="42" t="s">
         <v>122</v>
       </c>
-      <c r="C38" s="7" t="s">
+      <c r="C38" s="42" t="s">
         <v>123</v>
       </c>
     </row>
     <row r="39" spans="1:6" ht="45.6" x14ac:dyDescent="0.3">
-      <c r="A39" s="29" t="s">
+      <c r="A39" s="45" t="s">
         <v>24</v>
       </c>
-      <c r="B39" s="26" t="s">
+      <c r="B39" s="38" t="s">
         <v>94</v>
       </c>
-      <c r="C39" s="27" t="s">
+      <c r="C39" s="39" t="s">
         <v>95</v>
       </c>
-      <c r="D39" s="27" t="s">
+      <c r="D39" s="39" t="s">
         <v>124</v>
       </c>
-      <c r="E39" s="27" t="s">
+      <c r="E39" s="39" t="s">
         <v>97</v>
       </c>
-      <c r="F39" s="27" t="s">
+      <c r="F39" s="39" t="s">
         <v>98</v>
       </c>
     </row>
     <row r="40" spans="1:6" ht="57" x14ac:dyDescent="0.3">
-      <c r="A40" s="30" t="s">
+      <c r="A40" s="46" t="s">
         <v>30</v>
       </c>
-      <c r="B40" s="38" t="s">
+      <c r="B40" s="40" t="s">
         <v>99</v>
       </c>
-      <c r="C40" s="31" t="s">
+      <c r="C40" s="41" t="s">
         <v>100</v>
       </c>
-      <c r="D40" s="31" t="s">
+      <c r="D40" s="41" t="s">
         <v>125</v>
       </c>
-      <c r="E40" s="31" t="s">
+      <c r="E40" s="41" t="s">
         <v>102</v>
       </c>
-      <c r="F40" s="31" t="s">
+      <c r="F40" s="41" t="s">
         <v>103</v>
       </c>
     </row>
     <row r="41" spans="1:6" ht="57" x14ac:dyDescent="0.3">
-      <c r="A41" s="29" t="s">
+      <c r="A41" s="45" t="s">
         <v>37</v>
       </c>
-      <c r="B41" s="26" t="s">
+      <c r="B41" s="38" t="s">
         <v>94</v>
       </c>
-      <c r="C41" s="27" t="s">
+      <c r="C41" s="39" t="s">
         <v>126</v>
       </c>
-      <c r="D41" s="27" t="s">
+      <c r="D41" s="39" t="s">
         <v>127</v>
       </c>
-      <c r="E41" s="27" t="s">
+      <c r="E41" s="39" t="s">
         <v>128</v>
       </c>
-      <c r="F41" s="27" t="s">
+      <c r="F41" s="39" t="s">
         <v>129</v>
       </c>
     </row>
@@ -2731,20 +3034,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A1" s="45" t="s">
+      <c r="A1" s="34" t="s">
         <v>130</v>
       </c>
-      <c r="B1" s="44"/>
-      <c r="C1" s="44"/>
-      <c r="D1" s="44"/>
+      <c r="B1" s="35"/>
+      <c r="C1" s="35"/>
+      <c r="D1" s="35"/>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A2" s="49" t="s">
+      <c r="A2" s="37" t="s">
         <v>131</v>
       </c>
-      <c r="B2" s="44"/>
-      <c r="C2" s="44"/>
-      <c r="D2" s="44"/>
+      <c r="B2" s="35"/>
+      <c r="C2" s="35"/>
+      <c r="D2" s="35"/>
     </row>
     <row r="4" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
@@ -2772,10 +3075,10 @@
       <c r="B6" s="13" t="s">
         <v>138</v>
       </c>
-      <c r="C6" s="32" t="s">
+      <c r="C6" s="29" t="s">
         <v>139</v>
       </c>
-      <c r="D6" s="33" t="s">
+      <c r="D6" s="30" t="s">
         <v>188</v>
       </c>
     </row>
@@ -2786,10 +3089,10 @@
       <c r="B7" s="13" t="s">
         <v>141</v>
       </c>
-      <c r="C7" s="32" t="s">
+      <c r="C7" s="29" t="s">
         <v>139</v>
       </c>
-      <c r="D7" s="33" t="s">
+      <c r="D7" s="30" t="s">
         <v>189</v>
       </c>
     </row>
@@ -2800,10 +3103,10 @@
       <c r="B8" s="13" t="s">
         <v>143</v>
       </c>
-      <c r="C8" s="32" t="s">
+      <c r="C8" s="29" t="s">
         <v>139</v>
       </c>
-      <c r="D8" s="33" t="s">
+      <c r="D8" s="30" t="s">
         <v>144</v>
       </c>
     </row>
@@ -2814,10 +3117,10 @@
       <c r="B9" s="13" t="s">
         <v>146</v>
       </c>
-      <c r="C9" s="32" t="s">
+      <c r="C9" s="29" t="s">
         <v>139</v>
       </c>
-      <c r="D9" s="33" t="s">
+      <c r="D9" s="30" t="s">
         <v>221</v>
       </c>
     </row>
@@ -2828,10 +3131,10 @@
       <c r="B10" s="13" t="s">
         <v>148</v>
       </c>
-      <c r="C10" s="32" t="s">
+      <c r="C10" s="29" t="s">
         <v>139</v>
       </c>
-      <c r="D10" s="33" t="s">
+      <c r="D10" s="30" t="s">
         <v>222</v>
       </c>
     </row>
@@ -2861,10 +3164,10 @@
       <c r="B14" s="13" t="s">
         <v>151</v>
       </c>
-      <c r="C14" s="32" t="s">
+      <c r="C14" s="29" t="s">
         <v>139</v>
       </c>
-      <c r="D14" s="33" t="s">
+      <c r="D14" s="30" t="s">
         <v>190</v>
       </c>
     </row>
@@ -2875,10 +3178,10 @@
       <c r="B15" s="13" t="s">
         <v>152</v>
       </c>
-      <c r="C15" s="32" t="s">
+      <c r="C15" s="29" t="s">
         <v>139</v>
       </c>
-      <c r="D15" s="33" t="s">
+      <c r="D15" s="30" t="s">
         <v>191</v>
       </c>
     </row>
@@ -2889,10 +3192,10 @@
       <c r="B16" s="13" t="s">
         <v>153</v>
       </c>
-      <c r="C16" s="32" t="s">
+      <c r="C16" s="29" t="s">
         <v>139</v>
       </c>
-      <c r="D16" s="33" t="s">
+      <c r="D16" s="30" t="s">
         <v>154</v>
       </c>
     </row>
@@ -2903,10 +3206,10 @@
       <c r="B17" s="13" t="s">
         <v>155</v>
       </c>
-      <c r="C17" s="32" t="s">
+      <c r="C17" s="29" t="s">
         <v>139</v>
       </c>
-      <c r="D17" s="33" t="s">
+      <c r="D17" s="30" t="s">
         <v>156</v>
       </c>
     </row>
@@ -2917,10 +3220,10 @@
       <c r="B18" s="13" t="s">
         <v>157</v>
       </c>
-      <c r="C18" s="32" t="s">
+      <c r="C18" s="29" t="s">
         <v>139</v>
       </c>
-      <c r="D18" s="33" t="s">
+      <c r="D18" s="30" t="s">
         <v>158</v>
       </c>
     </row>
@@ -2967,13 +3270,13 @@
       <c r="A28" s="19" t="s">
         <v>10</v>
       </c>
-      <c r="B28" s="34" t="s">
+      <c r="B28" s="31" t="s">
         <v>167</v>
       </c>
-      <c r="C28" s="34" t="s">
+      <c r="C28" s="31" t="s">
         <v>168</v>
       </c>
-      <c r="D28" s="33" t="s">
+      <c r="D28" s="30" t="s">
         <v>186</v>
       </c>
     </row>
@@ -2981,13 +3284,13 @@
       <c r="A29" s="19" t="s">
         <v>13</v>
       </c>
-      <c r="B29" s="34" t="s">
+      <c r="B29" s="31" t="s">
         <v>169</v>
       </c>
-      <c r="C29" s="34" t="s">
+      <c r="C29" s="31" t="s">
         <v>170</v>
       </c>
-      <c r="D29" s="33" t="s">
+      <c r="D29" s="30" t="s">
         <v>171</v>
       </c>
     </row>
@@ -2995,13 +3298,13 @@
       <c r="A30" s="19" t="s">
         <v>16</v>
       </c>
-      <c r="B30" s="34" t="s">
+      <c r="B30" s="31" t="s">
         <v>172</v>
       </c>
-      <c r="C30" s="34" t="s">
+      <c r="C30" s="31" t="s">
         <v>173</v>
       </c>
-      <c r="D30" s="33" t="s">
+      <c r="D30" s="30" t="s">
         <v>186</v>
       </c>
     </row>
@@ -3009,13 +3312,13 @@
       <c r="A31" s="19" t="s">
         <v>18</v>
       </c>
-      <c r="B31" s="34" t="s">
+      <c r="B31" s="31" t="s">
         <v>174</v>
       </c>
-      <c r="C31" s="34" t="s">
+      <c r="C31" s="31" t="s">
         <v>175</v>
       </c>
-      <c r="D31" s="33" t="s">
+      <c r="D31" s="30" t="s">
         <v>176</v>
       </c>
     </row>
@@ -3023,13 +3326,13 @@
       <c r="A32" s="19" t="s">
         <v>24</v>
       </c>
-      <c r="B32" s="34" t="s">
+      <c r="B32" s="31" t="s">
         <v>177</v>
       </c>
-      <c r="C32" s="34" t="s">
+      <c r="C32" s="31" t="s">
         <v>178</v>
       </c>
-      <c r="D32" s="33" t="s">
+      <c r="D32" s="30" t="s">
         <v>179</v>
       </c>
     </row>
@@ -3037,13 +3340,13 @@
       <c r="A33" s="19" t="s">
         <v>30</v>
       </c>
-      <c r="B33" s="34" t="s">
+      <c r="B33" s="31" t="s">
         <v>180</v>
       </c>
-      <c r="C33" s="34" t="s">
+      <c r="C33" s="31" t="s">
         <v>181</v>
       </c>
-      <c r="D33" s="33" t="s">
+      <c r="D33" s="30" t="s">
         <v>182</v>
       </c>
     </row>
@@ -3051,13 +3354,13 @@
       <c r="A34" s="19" t="s">
         <v>37</v>
       </c>
-      <c r="B34" s="34" t="s">
+      <c r="B34" s="31" t="s">
         <v>183</v>
       </c>
-      <c r="C34" s="34" t="s">
+      <c r="C34" s="31" t="s">
         <v>184</v>
       </c>
-      <c r="D34" s="33" t="s">
+      <c r="D34" s="30" t="s">
         <v>185</v>
       </c>
     </row>

</xml_diff>